<commit_message>
Add Owner column to all_notifications_updated.xlsx, split evenly
First 64 rows assigned to Donte, remaining 64 to Samyukta.
</commit_message>
<xml_diff>
--- a/servicenow/email_notifications/all_notifications_updated.xlsx
+++ b/servicenow/email_notifications/all_notifications_updated.xlsx
@@ -456,12 +456,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="40" customWidth="1" style="1" min="1" max="1"/>
     <col width="12" customWidth="1" style="1" min="2" max="2"/>
     <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,6 +481,11 @@
           <t>Updated HTML</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="409.5" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
@@ -498,6 +504,11 @@
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;You have been mentioned&lt;/h1&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:ng_activity_mention_body}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -543,6 +554,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:manager_cc_not_vip}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="28.8" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -551,6 +567,11 @@
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.6" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -559,6 +580,11 @@
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="409.5" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -579,6 +605,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Approval reply not processed&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:approval_error_response}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -626,6 +657,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${approver},&lt;/p&gt;
 &lt;!-- 2-column tabular content --&gt;
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 0 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.short_description}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Click here to view Approval Request:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${URI}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Click here to view ${sysapproval.sys_class_name}:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.URI}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Priority:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.priority}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Category:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.category}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -743,6 +779,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="409.5" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
@@ -824,6 +865,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.short_description}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;On Behalf Of:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.request.requested_for}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.description}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;!-- 2-column tabular content --&gt;
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 0 0;" width="100%"&gt;&lt;tr&gt;&lt;td colspan="2" style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;Additional Details:&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Item Name:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.cat_item}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Opened:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.opened_at}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Opened By:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.opened_by}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Cube Location:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${sysapproval.request.requested_for.u_building}.${sysapproval.request.requested_for.u_cube}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -899,6 +945,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="409.5" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
@@ -1017,6 +1068,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="409.5" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
@@ -1138,6 +1194,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_isvcert_dl_to_cc}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="409.5" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
@@ -1191,6 +1252,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For any questions, please contact the EngSec team at &lt;a href="mailto:Eng-InfoSec-Support@exchange.nvidia.com" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;Eng-InfoSec-Support@exchange.nvidia.com&lt;/a&gt;.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="409.5" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
@@ -1221,6 +1287,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="409.5" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
@@ -1251,6 +1322,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="409.5" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
@@ -1280,6 +1356,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;To submit a new request, please &lt;a href="/esc?id=sc_cat_item&amp;amp;sys_id=255e97b1736610107e88ef66fbf6a7e3" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;click here&lt;/a&gt;. For any questions, please contact us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="43.2" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
@@ -1288,6 +1369,11 @@
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="409.5" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
@@ -1405,6 +1491,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="409.5" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
@@ -1428,6 +1519,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi ${requested_by},&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;The change request ${number} you requested has been taken off hold and is in the ${state} state.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Click here to view your change request: ${mail_script:nvidia_uri_ref_styled}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -1455,6 +1551,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;The change request ${number} you requested has been put on hold. The reason for the request being put on hold is:&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${on_hold_reason}&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Click here to view your change request: ${mail_script:nvidia_uri_ref_styled}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -1495,6 +1596,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="409.5" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
@@ -1519,6 +1625,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="259.2" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
@@ -1534,6 +1645,11 @@
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>&lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:cim_cancel_email}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -1595,6 +1711,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions or believe this request was made in error, please contact us in the #ask-cloud-desktop Slack channel.&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Thank you,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -1702,6 +1823,11 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="409.5" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -1807,6 +1933,11 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="409.5" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
@@ -1868,6 +1999,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="409.5" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
@@ -1908,6 +2044,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:Nvidia View Record}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="409.5" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -1931,6 +2072,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:sn_oe_sfs.collab_chat_new_member}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="409.5" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
@@ -1952,6 +2098,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;New unread messages&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:collaboration_direct_message_body}&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:collaboration_message_parser}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2051,6 +2202,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="409.5" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
@@ -2080,6 +2236,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Do not reply to this email, as this inbox is not monitored.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="409.5" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
@@ -2130,6 +2291,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;New Contingent Worker&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${name}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Hiring Manager&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_onboarding_manager}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_onboarding_hire_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Work Location&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_onboarding_location}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For questions, contact ${u_onboarding_manager}.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_manager_in_cc}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2165,6 +2331,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;&lt;em&gt;This is an AI Generated response. Please review for accuracy.&lt;/em&gt;&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="409.5" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
@@ -2215,6 +2386,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 0 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Name&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${name}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Display name&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${display_name}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Model number&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${model_number}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Normalization status&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${normalized_status}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Standard IT offering&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_standard_it_offering}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="331.2" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
@@ -2232,6 +2408,11 @@
         <is>
           <t>&lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi Team,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:duplicateOnboardingRITMs}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2301,6 +2482,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For any issues, please contact the Deemed Export team at &lt;a href="mailto:nvidia-deemedexport@nvidia.com" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;nvidia-deemedexport@nvidia.com&lt;/a&gt;.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="409.5" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
@@ -2332,6 +2518,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Service Request Number: ${mail_script:nvidia_ritm_number_link}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="409.5" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
@@ -2357,6 +2548,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;2. Sign in with your NVIDIA credentials. &lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For more details, click &lt;a href="/esc?id=kb_article&amp;amp;sysparm_article=KB0017080" style="color: #76b900; font-weight: bold; text-decoration: underline;"&gt;here&lt;/a&gt;.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you encounter issues during installation or ${mail_script:sc_req_item_request_fullfilled_adobe}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2386,6 +2582,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;You already have access to Google Drive. Sign in &lt;a href="https://drive.google.com/" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;here&lt;/a&gt; with your NVIDIA credentials.&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For more details, click &lt;a href="/esc?id=kb_article&amp;amp;sysparm_article=KB0017080" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;here&lt;/a&gt;.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you encounter issues during installation or ${mail_script:sc_req_item_request_fullfilled_adobe}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2433,6 +2634,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 0 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Number&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${URI_REF}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Coupa PR Number&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_requisition_id}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Coupa PO Numbers&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${mail_script:get_purchase_order_numbers}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="409.5" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
@@ -2477,6 +2683,11 @@
 &lt;!-- 2-column tabular content --&gt;
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Number:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${number}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Bulk Stock Records:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${mail_script:block_stock_records_link}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${short_description}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Coupa PR Number:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_requisition_id}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:Nvidia View Record}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2528,6 +2739,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 0 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Number&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${URI_REF}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${short_description}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Coupa PR Number&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_requisition_id}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Rejection Reason&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${event.parm2}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="409.5" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
@@ -2578,6 +2794,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:Nvidia View Record}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="409.5" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
@@ -2613,6 +2834,11 @@
 &lt;p style="margin: 0 0 8px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #000000; line-height: 1.5;"&gt;Request Details:&lt;/p&gt;
 &lt;!-- 2-column tabular content --&gt;
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 0 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Number:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${number}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Short Description:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${short_description}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -2726,6 +2952,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="409.5" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -2837,6 +3068,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="409.5" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
@@ -2948,6 +3184,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="409.5" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -2979,6 +3220,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="409.5" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
@@ -3002,6 +3248,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For proper IT Ticket categorization, the NVIDIA Help ticket you submitted ${request.parent.number}: ${request.parent.short_description} was automatically converted to ${number} and will be processed accordingly.&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Please refer to your new service request ${number} for status updates.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:Nvidia View Record}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -3037,6 +3288,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="409.5" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
@@ -3068,6 +3324,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="409.5" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
@@ -3093,6 +3354,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Incident ${mail_script:link_to_portal_nvidia} has been opened on your behalf.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="409.5" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
@@ -3118,6 +3384,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Incident ${mail_script:link_to_portal_nvidia} has been opened on your behalf.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="409.5" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
@@ -3143,6 +3414,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Incident ${mail_script:link_to_portal_nvidia} has been opened on your behalf.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="259.2" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
@@ -3165,6 +3441,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:incident_resolved_incident_details}&lt;/p&gt;
 &lt;!-- Tertiary CTA — link back to the ServiceNow platform --&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #76b900; line-height: 1.5;"&gt;${mail_script:incident_take_me_to_the_incident}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -3200,6 +3481,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Service Desk Team&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="409.5" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
@@ -3237,6 +3523,11 @@
 &lt;p style="margin: 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #76b900; line-height: 1.5;"&gt;${mail_script:incident_survey_link_nvidia}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="409.5" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
@@ -3268,6 +3559,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:incident_task_additional_details}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="409.5" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
@@ -3297,6 +3593,11 @@
 &lt;!-- Tertiary CTA — link back to the ServiceNow platform --&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #76b900; line-height: 1.5;"&gt;&lt;span data-teams="true"&gt;${mail_script:incident_task_take_me_to_the_incident}&lt;/span&gt;&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:incident_task_additional_details}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -3410,6 +3711,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="409.5" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
@@ -3448,6 +3754,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="57.6" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
@@ -3456,6 +3767,11 @@
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="409.5" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
@@ -3522,6 +3838,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;To cancel the loaner laptop request, access the ticket (${mail_script:add_link_to_loaner_asset_order}) and select the option to cancel the ticket. This will terminate the loaner process and close the request.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Donte</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="409.5" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
@@ -3586,6 +3907,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${return_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Pickup location:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;IT Tech Lounge at ${u_building}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us by updating the comments in ${mail_script:add_link_to_loaner_asset_order}.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;To cancel the loaner laptop request, access the ticket (${mail_script:add_link_to_loaner_asset_order}) and select the option to cancel the ticket. This will terminate the loaner process and close the request.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Donte</t>
         </is>
       </c>
     </row>
@@ -3623,6 +3949,11 @@
 &lt;li&gt;&lt;strong&gt;Review the Guide:&lt;/strong&gt; Follow the specific steps outlined in the &lt;a href="/kb_view.do?sysparm_article=KB0030680" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;GlobalProtect China User Guide&lt;/a&gt; to configure the connection correctly.&lt;/li&gt;
 &lt;li&gt;&lt;strong&gt;Pre-Trip Setup:&lt;/strong&gt; We strongly recommend verifying the configuration before departure.&lt;/li&gt;
 &lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -3695,6 +4026,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="409.5" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
@@ -3743,6 +4079,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Setting Up Your New Computer:&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Follow the &lt;a href="/esc?id=kb_article&amp;amp;sysparm_article=KB0027580" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;Windows&lt;/a&gt; or &lt;a href="/esc?id=kb_article&amp;amp;sysparm_article=KB0027581" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;Mac&lt;/a&gt; Setup Instructions document to provision your new computer.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Enjoy the new device!&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -3807,6 +4148,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Enjoy the new device!&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="409.5" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
@@ -3838,6 +4184,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Enjoy the new device!&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="409.5" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
@@ -3861,6 +4212,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Thank you for returning your device: ${mail_script:ITVM_reminder_mail_ritm_link}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="409.5" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
@@ -3884,6 +4240,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;This report list all employees that have multiple accessories, from the same type, assigned to them in the last year:  ${event.parm1}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="409.5" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
@@ -3905,6 +4266,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Multiple accessories from the same type&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello Team,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;This report list all employees that have multiple accessories, from the same type, assigned to them in the last year:  ${event.parm1}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -3945,6 +4311,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_global_trade_compliance_to_cc}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="409.5" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
@@ -3976,6 +4347,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:live_feed_message_headers}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="409.5" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
@@ -4030,6 +4406,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${loaner_order.u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${loaner_order.u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${loaner_order.start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${loaner_order.return_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Sensitive Loaner:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${loaner_order.u_sensitive_loaner}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_travel_loaner_sensitive_guides}&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us by updating the comments in ${mail_script:add_link_to_loaner_number}.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4077,6 +4458,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Comments: &lt;span data-teams="true"&gt;${mail_script:it_single_comment}&lt;/span&gt; &lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="409.5" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
@@ -4104,6 +4490,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us by updating the comments in ${mail_script:add_link_to_loaner_asset_order_reclam}.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="409.5" customHeight="1">
       <c r="A79" s="1" t="inlineStr">
@@ -4158,6 +4549,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${return_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Sensitive Loaner:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_sensitive_loaner}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_travel_loaner_sensitive_guides}&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us by updating the comments in ${mail_script:add_link_to_loaner_asset_order_reclam}.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4216,6 +4612,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="409.5" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
@@ -4243,6 +4644,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:return_loaner_instruction_ship_us}&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have already completed the return, please click ${mailto:mailto.confirm} to confirm the action. We apologize for any inconvenience. Thank you for the cooperation.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via ${mail_script:add_link_to_loaner_asset_order_reclam}.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4311,6 +4717,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_manager_hierarchy_cc_loaner}${mail_script:loaner_reminder_set_subject}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="409.5" customHeight="1">
       <c r="A83" s="1" t="inlineStr">
@@ -4377,6 +4788,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_manager_hierarchy_cc_loaner}${mail_script:loaner_reminder_set_subject}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="409.5" customHeight="1">
       <c r="A84" s="1" t="inlineStr">
@@ -4398,6 +4814,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Loaner reclaim closed&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${requested_for.first_name},&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Thank you for returning the loaner device: ${mail_script:add_link_to_loaner_asset_order_reclam}.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4456,6 +4877,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:loaner_cc_Assigned_to}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="409.5" customHeight="1">
       <c r="A86" s="1" t="inlineStr">
@@ -4506,6 +4932,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${return_date}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_manager_hierarchy_cc_loaner}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4562,6 +4993,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:loaner_cc_Assigned_to}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="409.5" customHeight="1">
       <c r="A88" s="1" t="inlineStr">
@@ -4618,6 +5054,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:loaner_cc_Assigned_to}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="409.5" customHeight="1">
       <c r="A89" s="1" t="inlineStr">
@@ -4668,6 +5109,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${return_date}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:loaner_cc_Assigned_to}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4697,6 +5143,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="409.5" customHeight="1">
       <c r="A91" s="1" t="inlineStr">
@@ -4720,6 +5171,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi ${user},&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${board.owner} has added you to the ${board.name} Visual Task Board.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;You can access the board &lt;a href="/$vtb.do?sysparm_board=${board.sys_id}" style="color: #76b900; font-weight: bold; text-decoration: underline;"&gt;${board.name}&lt;/a&gt; directly or via the Visual Task Board &lt;a href="/$vtb.do" style="color: #76b900; font-weight: bold; text-decoration: underline;"&gt;home page&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4747,6 +5203,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello ${requested_for},&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Your Microsoft Copilot license request has been successfully processed. Copilot will be activated for your account within the next 24-48 hours.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;To get started, visit our &lt;a href="https://nvidia.sharepoint.com/sites/MSTeams/SitePages/Microsoft-365-Copilot.aspx?xsdata=MDV8MDJ8fGJlOTBhNmM1NjA0YTQ0MmM3YjFkMDhkYzI4YWNmNjJifDQzMDgzZDE1NzI3MzQwYzFiN2RiMzllZmQ5Y2NjMTdhfDB8MHw2Mzg0Mjk5NzA1MDkyOTg0NjF8VW5rbm93bnxWR1ZoYlhOVFpXTjFjbWwwZVZObGNuWnBZMlY4ZXlKV0lqb2lNQzR3TGpBd01EQWlMQ0pRSWpvaVYybHVNeklpTENKQlRpSTZJazkwYUdWeUlpd2lWMVFpT2pFeGZRPT18MXxMMk5vWVhSekx6RTVPbTFsWlhScGJtZGZXV3BWZDFreVVURmFWRVYwVG5wS2FVNVRNREJQUjFwdFRGUnJNVTR5VVhST1IxRjNUVVJOTVU1WFNYZGFha1pyUUhSb2NtVmhaQzUyTWk5dFpYTnpZV2RsY3k4eE56QTNOREF3TWpRNU5qTTF8N2Q4NTUxOGJhZThmNDY5MDdiMWQwOGRjMjhhY2Y2MmJ8ZDI2NGM4MDIwNTM5NGRkY2JhODMwMzhlY2EzOWU2N2U%3D&amp;amp;sdata=RHBwSERCSEhVYklwZWV0QVhWUmJhcldnVlNEMEZwWTgrOTkrVXNuS0tMMD0%3D&amp;amp;ovuser=43083d15-7273-40c1-b7db-39efd9ccc17a%2Czriverasalas%40nvidia.com" rel="noopener noreferrer nofollow" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;SharePoint page&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4790,6 +5251,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you encounter issues during installation or ${mail_script:sc_req_item_request_fullfilled_adobe}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="409.5" customHeight="1">
       <c r="A94" s="1" t="inlineStr">
@@ -4821,6 +5287,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:sc_req_item_nv_refresh_ship_subject}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="409.5" customHeight="1">
       <c r="A95" s="1" t="inlineStr">
@@ -4840,6 +5311,11 @@
           <t>&lt;!-- Email Heading --&gt;
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Your one-time password&lt;/h1&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:multifactor_otp_email_notification}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -4897,6 +5373,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="409.5" customHeight="1">
       <c r="A97" s="1" t="inlineStr">
@@ -4929,6 +5410,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="409.5" customHeight="1">
       <c r="A98" s="1" t="inlineStr">
@@ -4954,6 +5440,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Our records shows that your new ${event.parm1} has been delivered. If that’s not the case or you are having issues with new ${event.parm1} or setup, please open an ${mail_script:create_incident_device_delivered}.&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Products being shipped to you&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:shipment_details_zt}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5018,6 +5509,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For any other questions, please add a comment to your ticket here: ${mail_script:laptop_desktop_proactive_refresh_ritm_link}&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Enjoy the new device!&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:set_subject_cc_for_asset_pickup}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5080,6 +5576,11 @@
 &lt;/ul&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; color: #000000; line-height: 1.5;"&gt;Setting up your new computer&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Follow the &lt;a href="/esc?id=kb_article&amp;amp;sysparm_article=KB0027580" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;Windows&lt;/a&gt; or &lt;a href="/esc?id=kb_article&amp;amp;sysparm_article=KB0027581" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;Mac&lt;/a&gt; Setup Instructions document to provision your new computer.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5205,6 +5706,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="409.5" customHeight="1">
       <c r="A102" s="1" t="inlineStr">
@@ -5322,6 +5828,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="409.5" customHeight="1">
       <c r="A103" s="1" t="inlineStr">
@@ -5380,6 +5891,11 @@
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${return_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Sensitive Loaner:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_sensitive_loaner}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;.&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:add_manager_hierarchy_cc_loaner}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5412,6 +5928,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:addProactiveUserstoBCC}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="409.5" customHeight="1">
       <c r="A105" s="1" t="inlineStr">
@@ -5433,6 +5954,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Your new computer is ready for pickup&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi ${requested_for},&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;We are pleased to inform you that the laptop is now ready to be picked up. Our Advanced Support team will reach out to you shortly with instructions on how to collect your laptop. We appreciate your patience and understanding.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5495,6 +6021,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:it_single_comment_clean}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="409.5" customHeight="1">
       <c r="A107" s="1" t="inlineStr">
@@ -5516,6 +6047,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;Export completed&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hello,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Please find the exported file ${attachment} attached to this email.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5559,6 +6095,11 @@
 &lt;li style="margin: 0 0 8px 0;"&gt;After setting up your new device, please drop off your old computer at the nearest ${mail_script:itvm_drop_asset_location}.&lt;/li&gt;
 &lt;/ol&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Enjoy the new device!&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5673,6 +6214,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="409.5" customHeight="1">
       <c r="A110" s="1" t="inlineStr">
@@ -5723,6 +6269,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:manager_cc_not_vip}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="409.5" customHeight="1">
       <c r="A111" s="1" t="inlineStr">
@@ -5753,6 +6304,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="409.5" customHeight="1">
       <c r="A112" s="1" t="inlineStr">
@@ -5781,6 +6337,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any feedback or if there are any issues with your order, we would appreciate your insights.&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Best Regards,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5851,6 +6412,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="409.5" customHeight="1">
       <c r="A114" s="1" t="inlineStr">
@@ -5897,6 +6463,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any feedback or if there are any issues with your order, we would appreciate your insights.&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Best Regards,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -5967,6 +6538,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;NVIDIA IT&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="409.5" customHeight="1">
       <c r="A116" s="1" t="inlineStr">
@@ -6008,6 +6584,11 @@
 &lt;li&gt;Stop by any tech lounge and hand over your old computer to an IT tech. You're done!&lt;/li&gt;
 &lt;/ul&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any feedback or if there are any issues with your order, we would appreciate your insights.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -6063,6 +6644,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;For any questions, please contact the EngSec team at &lt;a href="mailto:Eng-InfoSec-Support@exchange.nvidia.com" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;Eng-InfoSec-Support@exchange.nvidia.com&lt;/a&gt;.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="409.5" customHeight="1">
       <c r="A118" s="1" t="inlineStr">
@@ -6119,6 +6705,11 @@
 &lt;!-- 2-column tabular content --&gt;
 &lt;table border="0" cellpadding="0" cellspacing="0" role="presentation" style="margin: 0 0 24px 0;" width="100%"&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Loaner Type:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_loaner_type}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;OS:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_os_needed}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Start Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${start_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Return Date:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${return_date}&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 20px 8px 0; vertical-align: top; white-space: nowrap;"&gt;Sensitive Loaner:&lt;/td&gt;&lt;td style="font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; padding: 0 0 8px 0; vertical-align: top;"&gt;${u_sensitive_loaner}&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you have any questions, please reach out to us via &lt;a href="/esc" rel="noopener" style="color: #76b900; font-weight: bold; text-decoration: underline;" target="_blank"&gt;NVIDIA Help&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -6214,6 +6805,11 @@
         &lt;![endif]--&gt;&lt;!--[if !mso]&gt;&lt;!--&gt; &lt;a style="display: inline-block; background-color: #ffffff; color: #76b900; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: bold; text-decoration: none; padding: 11px 27px; border-radius: 6px; border: 1px solid #76b900; mso-hide: all;" href="${mailto_url:mailto.rejection}"&gt;&lt;span style="color: #76b900;"&gt;Reject&lt;/span&gt;&lt;/a&gt; &lt;!--&lt;![endif]--&gt;&lt;/td&gt;&lt;/tr&gt;
 &lt;/tbody&gt;
 &lt;/table&gt;</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -6324,6 +6920,11 @@
 &lt;/table&gt;</t>
         </is>
       </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="409.5" customHeight="1">
       <c r="A121" s="1" t="inlineStr">
@@ -6345,6 +6946,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:Nvidia View Record}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="43.2" customHeight="1">
       <c r="A122" s="1" t="inlineStr">
@@ -6353,6 +6959,11 @@
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr"/>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="409.5" customHeight="1">
       <c r="A123" s="1" t="inlineStr">
@@ -6461,6 +7072,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Thank you for your cooperation in keeping NVIDIA compliant while traveling.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="409.5" customHeight="1">
       <c r="A124" s="1" t="inlineStr">
@@ -6537,6 +7153,11 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="409.5" customHeight="1">
       <c r="A125" s="1" t="inlineStr">
@@ -6558,6 +7179,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;New message on Sidebar Discussion&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi ${name},&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:sidebar_discussion_reminder}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -6592,6 +7218,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Thank you! Looking forward to your response.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="409.5" customHeight="1">
       <c r="A127" s="1" t="inlineStr">
@@ -6619,6 +7250,11 @@
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Please review the details below:&lt;/p&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${mail_script:sws_multi_row_information}&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Have a great day.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>
@@ -6652,6 +7288,11 @@
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;If you encounter issues or ${mail_script:sc_req_item_request_fullfilled_adobe}&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="409.5" customHeight="1">
       <c r="A129" s="1" t="inlineStr">
@@ -6673,6 +7314,11 @@
 &lt;h1 style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 24px; font-weight: bold; color: #000000; line-height: 1.3;"&gt;${number} has been submitted&lt;/h1&gt;
 &lt;p style="margin: 0 0 24px 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;Hi,&lt;/p&gt;
 &lt;p style="margin: 0 0 0 0; font-family: 'NVIDIA Sans', 'Helvetica Neue', Helvetica, Arial, sans-serif; font-size: 16px; font-weight: 400; color: #000000; line-height: 1.5;"&gt;${short_description}&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Samyukta</t>
         </is>
       </c>
     </row>

</xml_diff>